<commit_message>
feat: finalize stage9 parity, add real-spec batch runner, and API/CLI bridge wiring
</commit_message>
<xml_diff>
--- a/rules/JABIL_X12_315_4010_to_JSON_TMSCARRIERTENDERRESPONSE_v1.4.xlsx
+++ b/rules/JABIL_X12_315_4010_to_JSON_TMSCARRIERTENDERRESPONSE_v1.4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnordin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A7F9164-E563-478B-8068-9B4809822D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="160" documentId="8_{90EE7985-014C-450F-9C1B-276C92E205A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0695638-543C-41AD-A2B2-9AF4893EBBB4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="818" xr2:uid="{610106AC-646B-484C-809A-4FBB47571196}"/>
   </bookViews>
@@ -1970,6 +1970,168 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1979,16 +2141,73 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1999,225 +2218,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2909,22 +2909,22 @@
       <c r="L1" s="71"/>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="154" t="s">
+      <c r="A2" s="163" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="155"/>
-      <c r="C2" s="155"/>
-      <c r="D2" s="155"/>
-      <c r="E2" s="155"/>
-      <c r="F2" s="156"/>
+      <c r="B2" s="164"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="165"/>
       <c r="G2" s="2"/>
       <c r="H2" s="63"/>
-      <c r="I2" s="163" t="s">
+      <c r="I2" s="169" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="164"/>
-      <c r="K2" s="164"/>
-      <c r="L2" s="165"/>
+      <c r="J2" s="170"/>
+      <c r="K2" s="170"/>
+      <c r="L2" s="171"/>
     </row>
     <row r="3" spans="1:14" ht="20.100000000000001">
       <c r="A3" s="64" t="s">
@@ -2965,7 +2965,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="9" customFormat="1">
-      <c r="A4" s="157" t="s">
+      <c r="A4" s="166" t="s">
         <v>22</v>
       </c>
       <c r="B4" s="38"/>
@@ -2985,7 +2985,7 @@
       <c r="L4" s="44"/>
     </row>
     <row r="5" spans="1:14" s="9" customFormat="1">
-      <c r="A5" s="158"/>
+      <c r="A5" s="167"/>
       <c r="B5" s="11"/>
       <c r="C5" s="46" t="s">
         <v>24</v>
@@ -3005,7 +3005,7 @@
       <c r="N5" s="8"/>
     </row>
     <row r="6" spans="1:14" s="9" customFormat="1" ht="64.5">
-      <c r="A6" s="158"/>
+      <c r="A6" s="167"/>
       <c r="B6" s="35" t="s">
         <v>26</v>
       </c>
@@ -3029,7 +3029,7 @@
       <c r="L6" s="8"/>
     </row>
     <row r="7" spans="1:14" s="13" customFormat="1" ht="30">
-      <c r="A7" s="158"/>
+      <c r="A7" s="167"/>
       <c r="B7" s="8" t="s">
         <v>31</v>
       </c>
@@ -3055,7 +3055,7 @@
       <c r="L7" s="7"/>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="158"/>
+      <c r="A8" s="167"/>
       <c r="B8" s="8" t="s">
         <v>0</v>
       </c>
@@ -3077,7 +3077,7 @@
       <c r="L8" s="12"/>
     </row>
     <row r="9" spans="1:14" s="9" customFormat="1" ht="10.5">
-      <c r="A9" s="158"/>
+      <c r="A9" s="167"/>
       <c r="B9" s="11" t="s">
         <v>38</v>
       </c>
@@ -3101,7 +3101,7 @@
       <c r="L9" s="8"/>
     </row>
     <row r="10" spans="1:14" s="13" customFormat="1" ht="10.5">
-      <c r="A10" s="158"/>
+      <c r="A10" s="167"/>
       <c r="B10" s="8" t="s">
         <v>41</v>
       </c>
@@ -3123,7 +3123,7 @@
       <c r="L10" s="7"/>
     </row>
     <row r="11" spans="1:14" s="13" customFormat="1" ht="50.1">
-      <c r="A11" s="158"/>
+      <c r="A11" s="167"/>
       <c r="B11" s="8" t="s">
         <v>44</v>
       </c>
@@ -3147,7 +3147,7 @@
       <c r="L11" s="18"/>
     </row>
     <row r="12" spans="1:14" ht="21.75">
-      <c r="A12" s="158"/>
+      <c r="A12" s="167"/>
       <c r="B12" s="8" t="s">
         <v>47</v>
       </c>
@@ -3169,7 +3169,7 @@
       <c r="L12" s="19"/>
     </row>
     <row r="13" spans="1:14" ht="42.75">
-      <c r="A13" s="158"/>
+      <c r="A13" s="167"/>
       <c r="B13" s="97" t="s">
         <v>51</v>
       </c>
@@ -3193,7 +3193,7 @@
       <c r="L13" s="19"/>
     </row>
     <row r="14" spans="1:14" ht="86.25">
-      <c r="A14" s="158"/>
+      <c r="A14" s="167"/>
       <c r="B14" s="8" t="s">
         <v>55</v>
       </c>
@@ -3217,7 +3217,7 @@
       <c r="L14" s="12"/>
     </row>
     <row r="15" spans="1:14">
-      <c r="A15" s="158"/>
+      <c r="A15" s="167"/>
       <c r="B15" s="8" t="s">
         <v>59</v>
       </c>
@@ -3239,7 +3239,7 @@
       <c r="L15" s="8"/>
     </row>
     <row r="16" spans="1:14">
-      <c r="A16" s="158"/>
+      <c r="A16" s="167"/>
       <c r="B16" s="8" t="s">
         <v>62</v>
       </c>
@@ -3261,7 +3261,7 @@
       <c r="L16" s="7"/>
     </row>
     <row r="17" spans="1:12" ht="10.5">
-      <c r="A17" s="158"/>
+      <c r="A17" s="167"/>
       <c r="B17" s="8" t="s">
         <v>64</v>
       </c>
@@ -3285,7 +3285,7 @@
       <c r="L17" s="8"/>
     </row>
     <row r="18" spans="1:12" ht="10.5">
-      <c r="A18" s="159"/>
+      <c r="A18" s="168"/>
       <c r="B18" s="8" t="s">
         <v>67</v>
       </c>
@@ -3309,7 +3309,7 @@
       <c r="L18" s="7"/>
     </row>
     <row r="19" spans="1:12" s="9" customFormat="1">
-      <c r="A19" s="160" t="s">
+      <c r="A19" s="119" t="s">
         <v>70</v>
       </c>
       <c r="B19" s="38"/>
@@ -3329,8 +3329,8 @@
       <c r="L19" s="44"/>
     </row>
     <row r="20" spans="1:12" ht="96.75">
-      <c r="A20" s="161"/>
-      <c r="B20" s="166" t="s">
+      <c r="A20" s="120"/>
+      <c r="B20" s="131" t="s">
         <v>71</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -3353,8 +3353,8 @@
       <c r="L20" s="8"/>
     </row>
     <row r="21" spans="1:12" ht="10.5">
-      <c r="A21" s="161"/>
-      <c r="B21" s="167"/>
+      <c r="A21" s="120"/>
+      <c r="B21" s="132"/>
       <c r="C21" s="8" t="s">
         <v>27</v>
       </c>
@@ -3375,8 +3375,8 @@
       <c r="L21" s="7"/>
     </row>
     <row r="22" spans="1:12">
-      <c r="A22" s="161"/>
-      <c r="B22" s="167"/>
+      <c r="A22" s="120"/>
+      <c r="B22" s="132"/>
       <c r="C22" s="8" t="s">
         <v>27</v>
       </c>
@@ -3395,8 +3395,8 @@
       <c r="L22" s="12"/>
     </row>
     <row r="23" spans="1:12">
-      <c r="A23" s="161"/>
-      <c r="B23" s="167"/>
+      <c r="A23" s="120"/>
+      <c r="B23" s="132"/>
       <c r="C23" s="8" t="s">
         <v>27</v>
       </c>
@@ -3415,8 +3415,8 @@
       <c r="L23" s="8"/>
     </row>
     <row r="24" spans="1:12">
-      <c r="A24" s="161"/>
-      <c r="B24" s="167"/>
+      <c r="A24" s="120"/>
+      <c r="B24" s="132"/>
       <c r="C24" s="8" t="s">
         <v>27</v>
       </c>
@@ -3435,8 +3435,8 @@
       <c r="L24" s="7"/>
     </row>
     <row r="25" spans="1:12">
-      <c r="A25" s="161"/>
-      <c r="B25" s="167"/>
+      <c r="A25" s="120"/>
+      <c r="B25" s="132"/>
       <c r="C25" s="8" t="s">
         <v>27</v>
       </c>
@@ -3455,8 +3455,8 @@
       <c r="L25" s="12"/>
     </row>
     <row r="26" spans="1:12">
-      <c r="A26" s="161"/>
-      <c r="B26" s="167"/>
+      <c r="A26" s="120"/>
+      <c r="B26" s="132"/>
       <c r="C26" s="8" t="s">
         <v>27</v>
       </c>
@@ -3475,8 +3475,8 @@
       <c r="L26" s="8"/>
     </row>
     <row r="27" spans="1:12">
-      <c r="A27" s="162"/>
-      <c r="B27" s="168"/>
+      <c r="A27" s="121"/>
+      <c r="B27" s="133"/>
       <c r="C27" s="8" t="s">
         <v>27</v>
       </c>
@@ -3521,16 +3521,16 @@
       <c r="L28" s="12"/>
     </row>
     <row r="29" spans="1:12">
-      <c r="A29" s="160" t="s">
+      <c r="A29" s="119" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="143" t="s">
+      <c r="B29" s="128" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="144"/>
-      <c r="D29" s="144"/>
-      <c r="E29" s="144"/>
-      <c r="F29" s="145"/>
+      <c r="C29" s="129"/>
+      <c r="D29" s="129"/>
+      <c r="E29" s="129"/>
+      <c r="F29" s="130"/>
       <c r="G29" s="51"/>
       <c r="H29" s="52" t="s">
         <v>23</v>
@@ -3541,11 +3541,11 @@
       <c r="L29" s="54"/>
     </row>
     <row r="30" spans="1:12" ht="21.75">
-      <c r="A30" s="161"/>
-      <c r="B30" s="166" t="s">
+      <c r="A30" s="120"/>
+      <c r="B30" s="131" t="s">
         <v>90</v>
       </c>
-      <c r="C30" s="149" t="s">
+      <c r="C30" s="156" t="s">
         <v>91</v>
       </c>
       <c r="D30" s="80" t="s">
@@ -3559,19 +3559,19 @@
       </c>
       <c r="G30" s="7"/>
       <c r="H30" s="31"/>
-      <c r="I30" s="129"/>
-      <c r="J30" s="119" t="s">
+      <c r="I30" s="176"/>
+      <c r="J30" s="173" t="s">
         <v>95</v>
       </c>
-      <c r="K30" s="119" t="s">
+      <c r="K30" s="173" t="s">
         <v>96</v>
       </c>
       <c r="L30" s="8"/>
     </row>
     <row r="31" spans="1:12" ht="9.9499999999999993" customHeight="1">
-      <c r="A31" s="161"/>
-      <c r="B31" s="167"/>
-      <c r="C31" s="125"/>
+      <c r="A31" s="120"/>
+      <c r="B31" s="132"/>
+      <c r="C31" s="157"/>
       <c r="D31" s="80" t="s">
         <v>97</v>
       </c>
@@ -3583,15 +3583,15 @@
       </c>
       <c r="G31" s="7"/>
       <c r="H31" s="31"/>
-      <c r="I31" s="130"/>
-      <c r="J31" s="120"/>
-      <c r="K31" s="125"/>
+      <c r="I31" s="177"/>
+      <c r="J31" s="174"/>
+      <c r="K31" s="157"/>
       <c r="L31" s="8"/>
     </row>
     <row r="32" spans="1:12" ht="9.9499999999999993" customHeight="1">
-      <c r="A32" s="161"/>
-      <c r="B32" s="167"/>
-      <c r="C32" s="125"/>
+      <c r="A32" s="120"/>
+      <c r="B32" s="132"/>
+      <c r="C32" s="157"/>
       <c r="D32" s="80" t="s">
         <v>100</v>
       </c>
@@ -3603,15 +3603,15 @@
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="31"/>
-      <c r="I32" s="130"/>
-      <c r="J32" s="121"/>
-      <c r="K32" s="124"/>
+      <c r="I32" s="177"/>
+      <c r="J32" s="175"/>
+      <c r="K32" s="172"/>
       <c r="L32" s="8"/>
     </row>
     <row r="33" spans="1:12" ht="18" customHeight="1">
-      <c r="A33" s="161"/>
-      <c r="B33" s="167"/>
-      <c r="C33" s="125"/>
+      <c r="A33" s="120"/>
+      <c r="B33" s="132"/>
+      <c r="C33" s="157"/>
       <c r="D33" s="80" t="s">
         <v>103</v>
       </c>
@@ -3623,19 +3623,19 @@
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="31"/>
-      <c r="I33" s="130"/>
-      <c r="J33" s="119" t="s">
+      <c r="I33" s="177"/>
+      <c r="J33" s="173" t="s">
         <v>106</v>
       </c>
-      <c r="K33" s="119" t="s">
+      <c r="K33" s="173" t="s">
         <v>107</v>
       </c>
       <c r="L33" s="8"/>
     </row>
     <row r="34" spans="1:12" ht="22.5" customHeight="1">
-      <c r="A34" s="161"/>
-      <c r="B34" s="167"/>
-      <c r="C34" s="125"/>
+      <c r="A34" s="120"/>
+      <c r="B34" s="132"/>
+      <c r="C34" s="157"/>
       <c r="D34" s="80" t="s">
         <v>108</v>
       </c>
@@ -3647,15 +3647,15 @@
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="31"/>
-      <c r="I34" s="130"/>
-      <c r="J34" s="124"/>
-      <c r="K34" s="124"/>
+      <c r="I34" s="177"/>
+      <c r="J34" s="172"/>
+      <c r="K34" s="172"/>
       <c r="L34" s="8"/>
     </row>
     <row r="35" spans="1:12" ht="20.100000000000001">
-      <c r="A35" s="161"/>
-      <c r="B35" s="167"/>
-      <c r="C35" s="124"/>
+      <c r="A35" s="120"/>
+      <c r="B35" s="132"/>
+      <c r="C35" s="172"/>
       <c r="D35" s="80" t="s">
         <v>110</v>
       </c>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="31"/>
-      <c r="I35" s="131"/>
+      <c r="I35" s="178"/>
       <c r="J35" s="75" t="s">
         <v>112</v>
       </c>
@@ -3675,9 +3675,9 @@
       <c r="L35" s="8"/>
     </row>
     <row r="36" spans="1:12">
-      <c r="A36" s="161"/>
-      <c r="B36" s="167"/>
-      <c r="C36" s="149" t="s">
+      <c r="A36" s="120"/>
+      <c r="B36" s="132"/>
+      <c r="C36" s="156" t="s">
         <v>91</v>
       </c>
       <c r="D36" s="80" t="s">
@@ -3691,15 +3691,15 @@
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="31"/>
-      <c r="I36" s="129"/>
-      <c r="J36" s="119"/>
-      <c r="K36" s="119"/>
+      <c r="I36" s="176"/>
+      <c r="J36" s="173"/>
+      <c r="K36" s="173"/>
       <c r="L36" s="7"/>
     </row>
     <row r="37" spans="1:12">
-      <c r="A37" s="161"/>
-      <c r="B37" s="167"/>
-      <c r="C37" s="125"/>
+      <c r="A37" s="120"/>
+      <c r="B37" s="132"/>
+      <c r="C37" s="157"/>
       <c r="D37" s="80" t="s">
         <v>115</v>
       </c>
@@ -3711,15 +3711,15 @@
       </c>
       <c r="G37" s="7"/>
       <c r="H37" s="31"/>
-      <c r="I37" s="130"/>
-      <c r="J37" s="125"/>
-      <c r="K37" s="125"/>
+      <c r="I37" s="177"/>
+      <c r="J37" s="157"/>
+      <c r="K37" s="157"/>
       <c r="L37" s="74"/>
     </row>
     <row r="38" spans="1:12">
-      <c r="A38" s="161"/>
-      <c r="B38" s="167"/>
-      <c r="C38" s="125"/>
+      <c r="A38" s="120"/>
+      <c r="B38" s="132"/>
+      <c r="C38" s="157"/>
       <c r="D38" s="80" t="s">
         <v>116</v>
       </c>
@@ -3731,15 +3731,15 @@
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="31"/>
-      <c r="I38" s="130"/>
-      <c r="J38" s="124"/>
-      <c r="K38" s="124"/>
+      <c r="I38" s="177"/>
+      <c r="J38" s="172"/>
+      <c r="K38" s="172"/>
       <c r="L38" s="74"/>
     </row>
     <row r="39" spans="1:12">
-      <c r="A39" s="161"/>
-      <c r="B39" s="167"/>
-      <c r="C39" s="125"/>
+      <c r="A39" s="120"/>
+      <c r="B39" s="132"/>
+      <c r="C39" s="157"/>
       <c r="D39" s="80" t="s">
         <v>117</v>
       </c>
@@ -3751,15 +3751,15 @@
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="31"/>
-      <c r="I39" s="130"/>
-      <c r="J39" s="151"/>
-      <c r="K39" s="119"/>
+      <c r="I39" s="177"/>
+      <c r="J39" s="179"/>
+      <c r="K39" s="173"/>
       <c r="L39" s="74"/>
     </row>
     <row r="40" spans="1:12">
-      <c r="A40" s="161"/>
-      <c r="B40" s="167"/>
-      <c r="C40" s="125"/>
+      <c r="A40" s="120"/>
+      <c r="B40" s="132"/>
+      <c r="C40" s="157"/>
       <c r="D40" s="80" t="s">
         <v>118</v>
       </c>
@@ -3771,15 +3771,15 @@
       </c>
       <c r="G40" s="7"/>
       <c r="H40" s="31"/>
-      <c r="I40" s="130"/>
-      <c r="J40" s="169"/>
-      <c r="K40" s="124"/>
+      <c r="I40" s="177"/>
+      <c r="J40" s="124"/>
+      <c r="K40" s="172"/>
       <c r="L40" s="74"/>
     </row>
     <row r="41" spans="1:12">
-      <c r="A41" s="161"/>
-      <c r="B41" s="167"/>
-      <c r="C41" s="124"/>
+      <c r="A41" s="120"/>
+      <c r="B41" s="132"/>
+      <c r="C41" s="172"/>
       <c r="D41" s="80" t="s">
         <v>119</v>
       </c>
@@ -3789,14 +3789,14 @@
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="31"/>
-      <c r="I41" s="131"/>
+      <c r="I41" s="178"/>
       <c r="J41" s="75"/>
       <c r="K41" s="10"/>
       <c r="L41" s="74"/>
     </row>
     <row r="42" spans="1:12">
-      <c r="A42" s="161"/>
-      <c r="B42" s="167"/>
+      <c r="A42" s="120"/>
+      <c r="B42" s="132"/>
       <c r="C42" s="78" t="s">
         <v>27</v>
       </c>
@@ -3815,9 +3815,9 @@
       <c r="L42" s="8"/>
     </row>
     <row r="43" spans="1:12">
-      <c r="A43" s="161"/>
-      <c r="B43" s="167"/>
-      <c r="C43" s="119" t="s">
+      <c r="A43" s="120"/>
+      <c r="B43" s="132"/>
+      <c r="C43" s="173" t="s">
         <v>91</v>
       </c>
       <c r="D43" s="80" t="s">
@@ -3831,15 +3831,15 @@
       </c>
       <c r="G43" s="83"/>
       <c r="H43" s="29"/>
-      <c r="I43" s="129"/>
-      <c r="J43" s="119"/>
-      <c r="K43" s="119"/>
+      <c r="I43" s="176"/>
+      <c r="J43" s="173"/>
+      <c r="K43" s="173"/>
       <c r="L43" s="83"/>
     </row>
     <row r="44" spans="1:12">
-      <c r="A44" s="161"/>
-      <c r="B44" s="167"/>
-      <c r="C44" s="120"/>
+      <c r="A44" s="120"/>
+      <c r="B44" s="132"/>
+      <c r="C44" s="174"/>
       <c r="D44" s="80" t="s">
         <v>122</v>
       </c>
@@ -3851,15 +3851,15 @@
       </c>
       <c r="G44" s="83"/>
       <c r="H44" s="29"/>
-      <c r="I44" s="130"/>
-      <c r="J44" s="120"/>
-      <c r="K44" s="120"/>
+      <c r="I44" s="177"/>
+      <c r="J44" s="174"/>
+      <c r="K44" s="174"/>
       <c r="L44" s="85"/>
     </row>
     <row r="45" spans="1:12">
-      <c r="A45" s="161"/>
-      <c r="B45" s="167"/>
-      <c r="C45" s="120"/>
+      <c r="A45" s="120"/>
+      <c r="B45" s="132"/>
+      <c r="C45" s="174"/>
       <c r="D45" s="80" t="s">
         <v>123</v>
       </c>
@@ -3871,15 +3871,15 @@
       </c>
       <c r="G45" s="83"/>
       <c r="H45" s="29"/>
-      <c r="I45" s="130"/>
-      <c r="J45" s="121"/>
-      <c r="K45" s="121"/>
+      <c r="I45" s="177"/>
+      <c r="J45" s="175"/>
+      <c r="K45" s="175"/>
       <c r="L45" s="85"/>
     </row>
     <row r="46" spans="1:12">
-      <c r="A46" s="161"/>
-      <c r="B46" s="167"/>
-      <c r="C46" s="120"/>
+      <c r="A46" s="120"/>
+      <c r="B46" s="132"/>
+      <c r="C46" s="174"/>
       <c r="D46" s="80" t="s">
         <v>124</v>
       </c>
@@ -3891,15 +3891,15 @@
       </c>
       <c r="G46" s="83"/>
       <c r="H46" s="29"/>
-      <c r="I46" s="130"/>
-      <c r="J46" s="119"/>
-      <c r="K46" s="119"/>
+      <c r="I46" s="177"/>
+      <c r="J46" s="173"/>
+      <c r="K46" s="173"/>
       <c r="L46" s="85"/>
     </row>
     <row r="47" spans="1:12">
-      <c r="A47" s="161"/>
-      <c r="B47" s="167"/>
-      <c r="C47" s="120"/>
+      <c r="A47" s="120"/>
+      <c r="B47" s="132"/>
+      <c r="C47" s="174"/>
       <c r="D47" s="80" t="s">
         <v>125</v>
       </c>
@@ -3911,15 +3911,15 @@
       </c>
       <c r="G47" s="83"/>
       <c r="H47" s="29"/>
-      <c r="I47" s="130"/>
-      <c r="J47" s="121"/>
-      <c r="K47" s="121"/>
+      <c r="I47" s="177"/>
+      <c r="J47" s="175"/>
+      <c r="K47" s="175"/>
       <c r="L47" s="85"/>
     </row>
     <row r="48" spans="1:12">
-      <c r="A48" s="161"/>
-      <c r="B48" s="167"/>
-      <c r="C48" s="121"/>
+      <c r="A48" s="120"/>
+      <c r="B48" s="132"/>
+      <c r="C48" s="175"/>
       <c r="D48" s="80" t="s">
         <v>126</v>
       </c>
@@ -3929,14 +3929,14 @@
       </c>
       <c r="G48" s="83"/>
       <c r="H48" s="29"/>
-      <c r="I48" s="131"/>
+      <c r="I48" s="178"/>
       <c r="J48" s="75"/>
       <c r="K48" s="75"/>
       <c r="L48" s="85"/>
     </row>
     <row r="49" spans="1:12">
-      <c r="A49" s="161"/>
-      <c r="B49" s="167"/>
+      <c r="A49" s="120"/>
+      <c r="B49" s="132"/>
       <c r="C49" s="81"/>
       <c r="D49" s="80"/>
       <c r="E49" s="82"/>
@@ -3949,8 +3949,8 @@
       <c r="L49" s="85"/>
     </row>
     <row r="50" spans="1:12">
-      <c r="A50" s="161"/>
-      <c r="B50" s="167"/>
+      <c r="A50" s="120"/>
+      <c r="B50" s="132"/>
       <c r="C50" s="8" t="s">
         <v>127</v>
       </c>
@@ -3969,8 +3969,8 @@
       <c r="L50" s="12"/>
     </row>
     <row r="51" spans="1:12">
-      <c r="A51" s="161"/>
-      <c r="B51" s="167"/>
+      <c r="A51" s="120"/>
+      <c r="B51" s="132"/>
       <c r="C51" s="48" t="s">
         <v>27</v>
       </c>
@@ -3989,8 +3989,8 @@
       <c r="L51" s="8"/>
     </row>
     <row r="52" spans="1:12">
-      <c r="A52" s="161"/>
-      <c r="B52" s="167"/>
+      <c r="A52" s="120"/>
+      <c r="B52" s="132"/>
       <c r="C52" s="48" t="s">
         <v>27</v>
       </c>
@@ -4009,8 +4009,8 @@
       <c r="L52" s="8"/>
     </row>
     <row r="53" spans="1:12">
-      <c r="A53" s="161"/>
-      <c r="B53" s="167"/>
+      <c r="A53" s="120"/>
+      <c r="B53" s="132"/>
       <c r="C53" s="48" t="s">
         <v>27</v>
       </c>
@@ -4029,8 +4029,8 @@
       <c r="L53" s="8"/>
     </row>
     <row r="54" spans="1:12">
-      <c r="A54" s="162"/>
-      <c r="B54" s="168"/>
+      <c r="A54" s="121"/>
+      <c r="B54" s="133"/>
       <c r="C54" s="48" t="s">
         <v>27</v>
       </c>
@@ -4049,16 +4049,16 @@
       <c r="L54" s="8"/>
     </row>
     <row r="55" spans="1:12" ht="10.5">
-      <c r="A55" s="160" t="s">
+      <c r="A55" s="119" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="143" t="s">
+      <c r="B55" s="128" t="s">
         <v>133</v>
       </c>
-      <c r="C55" s="144"/>
-      <c r="D55" s="144"/>
-      <c r="E55" s="144"/>
-      <c r="F55" s="145"/>
+      <c r="C55" s="129"/>
+      <c r="D55" s="129"/>
+      <c r="E55" s="129"/>
+      <c r="F55" s="130"/>
       <c r="G55" s="51"/>
       <c r="H55" s="52" t="s">
         <v>23</v>
@@ -4069,11 +4069,11 @@
       <c r="L55" s="54"/>
     </row>
     <row r="56" spans="1:12" ht="21.75">
-      <c r="A56" s="161"/>
-      <c r="B56" s="166" t="s">
+      <c r="A56" s="120"/>
+      <c r="B56" s="131" t="s">
         <v>90</v>
       </c>
-      <c r="C56" s="149" t="s">
+      <c r="C56" s="156" t="s">
         <v>91</v>
       </c>
       <c r="D56" s="80" t="s">
@@ -4087,19 +4087,19 @@
       </c>
       <c r="G56" s="18"/>
       <c r="H56" s="31"/>
-      <c r="I56" s="129"/>
-      <c r="J56" s="119" t="s">
+      <c r="I56" s="176"/>
+      <c r="J56" s="173" t="s">
         <v>95</v>
       </c>
-      <c r="K56" s="119" t="s">
+      <c r="K56" s="173" t="s">
         <v>96</v>
       </c>
       <c r="L56" s="8"/>
     </row>
     <row r="57" spans="1:12" ht="21.75">
-      <c r="A57" s="161"/>
-      <c r="B57" s="167"/>
-      <c r="C57" s="125"/>
+      <c r="A57" s="120"/>
+      <c r="B57" s="132"/>
+      <c r="C57" s="157"/>
       <c r="D57" s="80" t="s">
         <v>97</v>
       </c>
@@ -4111,15 +4111,15 @@
       </c>
       <c r="G57" s="18"/>
       <c r="H57" s="31"/>
-      <c r="I57" s="130"/>
-      <c r="J57" s="120"/>
-      <c r="K57" s="125"/>
+      <c r="I57" s="177"/>
+      <c r="J57" s="174"/>
+      <c r="K57" s="157"/>
       <c r="L57" s="8"/>
     </row>
     <row r="58" spans="1:12" ht="21.75">
-      <c r="A58" s="161"/>
-      <c r="B58" s="167"/>
-      <c r="C58" s="125"/>
+      <c r="A58" s="120"/>
+      <c r="B58" s="132"/>
+      <c r="C58" s="157"/>
       <c r="D58" s="80" t="s">
         <v>100</v>
       </c>
@@ -4131,15 +4131,15 @@
       </c>
       <c r="G58" s="18"/>
       <c r="H58" s="31"/>
-      <c r="I58" s="130"/>
-      <c r="J58" s="121"/>
-      <c r="K58" s="124"/>
+      <c r="I58" s="177"/>
+      <c r="J58" s="175"/>
+      <c r="K58" s="172"/>
       <c r="L58" s="8"/>
     </row>
     <row r="59" spans="1:12" ht="21.75">
-      <c r="A59" s="161"/>
-      <c r="B59" s="167"/>
-      <c r="C59" s="125"/>
+      <c r="A59" s="120"/>
+      <c r="B59" s="132"/>
+      <c r="C59" s="157"/>
       <c r="D59" s="80" t="s">
         <v>103</v>
       </c>
@@ -4151,19 +4151,19 @@
       </c>
       <c r="G59" s="18"/>
       <c r="H59" s="31"/>
-      <c r="I59" s="130"/>
-      <c r="J59" s="119" t="s">
+      <c r="I59" s="177"/>
+      <c r="J59" s="173" t="s">
         <v>106</v>
       </c>
-      <c r="K59" s="119" t="s">
+      <c r="K59" s="173" t="s">
         <v>107</v>
       </c>
       <c r="L59" s="8"/>
     </row>
     <row r="60" spans="1:12" ht="21.75">
-      <c r="A60" s="161"/>
-      <c r="B60" s="167"/>
-      <c r="C60" s="125"/>
+      <c r="A60" s="120"/>
+      <c r="B60" s="132"/>
+      <c r="C60" s="157"/>
       <c r="D60" s="80" t="s">
         <v>108</v>
       </c>
@@ -4175,15 +4175,15 @@
       </c>
       <c r="G60" s="18"/>
       <c r="H60" s="31"/>
-      <c r="I60" s="130"/>
-      <c r="J60" s="124"/>
-      <c r="K60" s="124"/>
+      <c r="I60" s="177"/>
+      <c r="J60" s="172"/>
+      <c r="K60" s="172"/>
       <c r="L60" s="8"/>
     </row>
     <row r="61" spans="1:12" ht="21.75">
-      <c r="A61" s="161"/>
-      <c r="B61" s="167"/>
-      <c r="C61" s="124"/>
+      <c r="A61" s="120"/>
+      <c r="B61" s="132"/>
+      <c r="C61" s="172"/>
       <c r="D61" s="80" t="s">
         <v>110</v>
       </c>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="G61" s="18"/>
       <c r="H61" s="31"/>
-      <c r="I61" s="130"/>
+      <c r="I61" s="177"/>
       <c r="J61" s="75" t="s">
         <v>112</v>
       </c>
@@ -4203,9 +4203,9 @@
       <c r="L61" s="8"/>
     </row>
     <row r="62" spans="1:12" ht="21.75">
-      <c r="A62" s="161"/>
-      <c r="B62" s="167"/>
-      <c r="C62" s="149" t="s">
+      <c r="A62" s="120"/>
+      <c r="B62" s="132"/>
+      <c r="C62" s="156" t="s">
         <v>91</v>
       </c>
       <c r="D62" s="80" t="s">
@@ -4219,19 +4219,19 @@
       </c>
       <c r="G62" s="90"/>
       <c r="H62" s="117"/>
-      <c r="I62" s="132"/>
-      <c r="J62" s="134" t="s">
+      <c r="I62" s="194"/>
+      <c r="J62" s="196" t="s">
         <v>95</v>
       </c>
-      <c r="K62" s="134" t="s">
+      <c r="K62" s="196" t="s">
         <v>96</v>
       </c>
       <c r="L62" s="8"/>
     </row>
     <row r="63" spans="1:12" ht="21.75">
-      <c r="A63" s="161"/>
-      <c r="B63" s="167"/>
-      <c r="C63" s="125"/>
+      <c r="A63" s="120"/>
+      <c r="B63" s="132"/>
+      <c r="C63" s="157"/>
       <c r="D63" s="80" t="s">
         <v>115</v>
       </c>
@@ -4243,15 +4243,15 @@
       </c>
       <c r="G63" s="90"/>
       <c r="H63" s="117"/>
-      <c r="I63" s="133"/>
-      <c r="J63" s="135"/>
-      <c r="K63" s="135"/>
+      <c r="I63" s="195"/>
+      <c r="J63" s="197"/>
+      <c r="K63" s="197"/>
       <c r="L63" s="8"/>
     </row>
     <row r="64" spans="1:12" ht="21.75">
-      <c r="A64" s="161"/>
-      <c r="B64" s="167"/>
-      <c r="C64" s="125"/>
+      <c r="A64" s="120"/>
+      <c r="B64" s="132"/>
+      <c r="C64" s="157"/>
       <c r="D64" s="80" t="s">
         <v>116</v>
       </c>
@@ -4263,15 +4263,15 @@
       </c>
       <c r="G64" s="90"/>
       <c r="H64" s="117"/>
-      <c r="I64" s="133"/>
-      <c r="J64" s="136"/>
-      <c r="K64" s="136"/>
+      <c r="I64" s="195"/>
+      <c r="J64" s="198"/>
+      <c r="K64" s="198"/>
       <c r="L64" s="8"/>
     </row>
     <row r="65" spans="1:12" ht="20.100000000000001" customHeight="1">
-      <c r="A65" s="161"/>
-      <c r="B65" s="167"/>
-      <c r="C65" s="125"/>
+      <c r="A65" s="120"/>
+      <c r="B65" s="132"/>
+      <c r="C65" s="157"/>
       <c r="D65" s="80" t="s">
         <v>117</v>
       </c>
@@ -4283,19 +4283,19 @@
       </c>
       <c r="G65" s="90"/>
       <c r="H65" s="117"/>
-      <c r="I65" s="133"/>
-      <c r="J65" s="134" t="s">
+      <c r="I65" s="195"/>
+      <c r="J65" s="196" t="s">
         <v>106</v>
       </c>
-      <c r="K65" s="134" t="s">
+      <c r="K65" s="196" t="s">
         <v>107</v>
       </c>
       <c r="L65" s="8"/>
     </row>
     <row r="66" spans="1:12" ht="20.100000000000001" customHeight="1">
-      <c r="A66" s="161"/>
-      <c r="B66" s="167"/>
-      <c r="C66" s="125"/>
+      <c r="A66" s="120"/>
+      <c r="B66" s="132"/>
+      <c r="C66" s="157"/>
       <c r="D66" s="80" t="s">
         <v>118</v>
       </c>
@@ -4307,15 +4307,15 @@
       </c>
       <c r="G66" s="90"/>
       <c r="H66" s="117"/>
-      <c r="I66" s="133"/>
-      <c r="J66" s="136"/>
-      <c r="K66" s="136"/>
+      <c r="I66" s="195"/>
+      <c r="J66" s="198"/>
+      <c r="K66" s="198"/>
       <c r="L66" s="8"/>
     </row>
     <row r="67" spans="1:12" ht="21.75">
-      <c r="A67" s="161"/>
-      <c r="B67" s="167"/>
-      <c r="C67" s="125"/>
+      <c r="A67" s="120"/>
+      <c r="B67" s="132"/>
+      <c r="C67" s="157"/>
       <c r="D67" s="80" t="s">
         <v>119</v>
       </c>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="G67" s="90"/>
       <c r="H67" s="117"/>
-      <c r="I67" s="133"/>
+      <c r="I67" s="195"/>
       <c r="J67" s="118" t="s">
         <v>112</v>
       </c>
@@ -4335,8 +4335,8 @@
       <c r="L67" s="8"/>
     </row>
     <row r="68" spans="1:12">
-      <c r="A68" s="161"/>
-      <c r="B68" s="167"/>
+      <c r="A68" s="120"/>
+      <c r="B68" s="132"/>
       <c r="C68" s="78" t="s">
         <v>27</v>
       </c>
@@ -4355,9 +4355,9 @@
       <c r="L68" s="8"/>
     </row>
     <row r="69" spans="1:12">
-      <c r="A69" s="161"/>
-      <c r="B69" s="167"/>
-      <c r="C69" s="119" t="s">
+      <c r="A69" s="120"/>
+      <c r="B69" s="132"/>
+      <c r="C69" s="173" t="s">
         <v>91</v>
       </c>
       <c r="D69" s="80" t="s">
@@ -4371,15 +4371,15 @@
       </c>
       <c r="G69" s="83"/>
       <c r="H69" s="29"/>
-      <c r="I69" s="129"/>
-      <c r="J69" s="119"/>
-      <c r="K69" s="119"/>
+      <c r="I69" s="176"/>
+      <c r="J69" s="173"/>
+      <c r="K69" s="173"/>
       <c r="L69" s="83"/>
     </row>
     <row r="70" spans="1:12">
-      <c r="A70" s="161"/>
-      <c r="B70" s="167"/>
-      <c r="C70" s="120"/>
+      <c r="A70" s="120"/>
+      <c r="B70" s="132"/>
+      <c r="C70" s="174"/>
       <c r="D70" s="80" t="s">
         <v>122</v>
       </c>
@@ -4391,15 +4391,15 @@
       </c>
       <c r="G70" s="83"/>
       <c r="H70" s="29"/>
-      <c r="I70" s="130"/>
-      <c r="J70" s="120"/>
-      <c r="K70" s="120"/>
+      <c r="I70" s="177"/>
+      <c r="J70" s="174"/>
+      <c r="K70" s="174"/>
       <c r="L70" s="85"/>
     </row>
     <row r="71" spans="1:12">
-      <c r="A71" s="161"/>
-      <c r="B71" s="167"/>
-      <c r="C71" s="120"/>
+      <c r="A71" s="120"/>
+      <c r="B71" s="132"/>
+      <c r="C71" s="174"/>
       <c r="D71" s="80" t="s">
         <v>123</v>
       </c>
@@ -4411,15 +4411,15 @@
       </c>
       <c r="G71" s="83"/>
       <c r="H71" s="29"/>
-      <c r="I71" s="130"/>
-      <c r="J71" s="121"/>
-      <c r="K71" s="121"/>
+      <c r="I71" s="177"/>
+      <c r="J71" s="175"/>
+      <c r="K71" s="175"/>
       <c r="L71" s="85"/>
     </row>
     <row r="72" spans="1:12">
-      <c r="A72" s="161"/>
-      <c r="B72" s="167"/>
-      <c r="C72" s="120"/>
+      <c r="A72" s="120"/>
+      <c r="B72" s="132"/>
+      <c r="C72" s="174"/>
       <c r="D72" s="80" t="s">
         <v>124</v>
       </c>
@@ -4431,15 +4431,15 @@
       </c>
       <c r="G72" s="83"/>
       <c r="H72" s="29"/>
-      <c r="I72" s="130"/>
-      <c r="J72" s="119"/>
-      <c r="K72" s="119"/>
+      <c r="I72" s="177"/>
+      <c r="J72" s="173"/>
+      <c r="K72" s="173"/>
       <c r="L72" s="85"/>
     </row>
     <row r="73" spans="1:12">
-      <c r="A73" s="161"/>
-      <c r="B73" s="167"/>
-      <c r="C73" s="120"/>
+      <c r="A73" s="120"/>
+      <c r="B73" s="132"/>
+      <c r="C73" s="174"/>
       <c r="D73" s="80" t="s">
         <v>125</v>
       </c>
@@ -4451,15 +4451,15 @@
       </c>
       <c r="G73" s="83"/>
       <c r="H73" s="29"/>
-      <c r="I73" s="130"/>
-      <c r="J73" s="121"/>
-      <c r="K73" s="121"/>
+      <c r="I73" s="177"/>
+      <c r="J73" s="175"/>
+      <c r="K73" s="175"/>
       <c r="L73" s="85"/>
     </row>
     <row r="74" spans="1:12">
-      <c r="A74" s="161"/>
-      <c r="B74" s="167"/>
-      <c r="C74" s="121"/>
+      <c r="A74" s="120"/>
+      <c r="B74" s="132"/>
+      <c r="C74" s="175"/>
       <c r="D74" s="80" t="s">
         <v>126</v>
       </c>
@@ -4469,14 +4469,14 @@
       </c>
       <c r="G74" s="83"/>
       <c r="H74" s="29"/>
-      <c r="I74" s="131"/>
+      <c r="I74" s="178"/>
       <c r="J74" s="75"/>
       <c r="K74" s="75"/>
       <c r="L74" s="85"/>
     </row>
     <row r="75" spans="1:12">
-      <c r="A75" s="161"/>
-      <c r="B75" s="167"/>
+      <c r="A75" s="120"/>
+      <c r="B75" s="132"/>
       <c r="C75" s="89"/>
       <c r="D75" s="86"/>
       <c r="E75" s="87"/>
@@ -4489,8 +4489,8 @@
       <c r="L75" s="93"/>
     </row>
     <row r="76" spans="1:12">
-      <c r="A76" s="161"/>
-      <c r="B76" s="167"/>
+      <c r="A76" s="120"/>
+      <c r="B76" s="132"/>
       <c r="C76" s="97" t="s">
         <v>135</v>
       </c>
@@ -4509,8 +4509,8 @@
       <c r="L76" s="12"/>
     </row>
     <row r="77" spans="1:12">
-      <c r="A77" s="161"/>
-      <c r="B77" s="167"/>
+      <c r="A77" s="120"/>
+      <c r="B77" s="132"/>
       <c r="C77" s="48" t="s">
         <v>27</v>
       </c>
@@ -4529,8 +4529,8 @@
       <c r="L77" s="8"/>
     </row>
     <row r="78" spans="1:12">
-      <c r="A78" s="161"/>
-      <c r="B78" s="167"/>
+      <c r="A78" s="120"/>
+      <c r="B78" s="132"/>
       <c r="C78" s="48" t="s">
         <v>27</v>
       </c>
@@ -4549,8 +4549,8 @@
       <c r="L78" s="8"/>
     </row>
     <row r="79" spans="1:12">
-      <c r="A79" s="161"/>
-      <c r="B79" s="167"/>
+      <c r="A79" s="120"/>
+      <c r="B79" s="132"/>
       <c r="C79" s="48" t="s">
         <v>27</v>
       </c>
@@ -4569,8 +4569,8 @@
       <c r="L79" s="8"/>
     </row>
     <row r="80" spans="1:12">
-      <c r="A80" s="162"/>
-      <c r="B80" s="168"/>
+      <c r="A80" s="121"/>
+      <c r="B80" s="133"/>
       <c r="C80" s="48" t="s">
         <v>27</v>
       </c>
@@ -4589,31 +4589,31 @@
       <c r="L80" s="19"/>
     </row>
     <row r="81" spans="1:12" s="21" customFormat="1" ht="10.5">
-      <c r="A81" s="188" t="s">
+      <c r="A81" s="147" t="s">
         <v>136</v>
       </c>
-      <c r="B81" s="191" t="s">
+      <c r="B81" s="150" t="s">
         <v>137</v>
       </c>
-      <c r="C81" s="192"/>
-      <c r="D81" s="192"/>
-      <c r="E81" s="192"/>
-      <c r="F81" s="193"/>
+      <c r="C81" s="151"/>
+      <c r="D81" s="151"/>
+      <c r="E81" s="151"/>
+      <c r="F81" s="152"/>
       <c r="G81" s="83"/>
       <c r="H81" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I81" s="194"/>
-      <c r="J81" s="195"/>
-      <c r="K81" s="195"/>
-      <c r="L81" s="196"/>
+      <c r="I81" s="153"/>
+      <c r="J81" s="154"/>
+      <c r="K81" s="154"/>
+      <c r="L81" s="155"/>
     </row>
     <row r="82" spans="1:12" s="21" customFormat="1" ht="20.100000000000001">
-      <c r="A82" s="189"/>
-      <c r="B82" s="153" t="s">
+      <c r="A82" s="148"/>
+      <c r="B82" s="191" t="s">
         <v>138</v>
       </c>
-      <c r="C82" s="123" t="s">
+      <c r="C82" s="192" t="s">
         <v>139</v>
       </c>
       <c r="D82" s="80" t="s">
@@ -4627,19 +4627,19 @@
       </c>
       <c r="G82" s="109"/>
       <c r="H82" s="110"/>
-      <c r="I82" s="150"/>
-      <c r="J82" s="119" t="s">
+      <c r="I82" s="189"/>
+      <c r="J82" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="K82" s="119" t="s">
+      <c r="K82" s="173" t="s">
         <v>143</v>
       </c>
-      <c r="L82" s="150"/>
+      <c r="L82" s="189"/>
     </row>
     <row r="83" spans="1:12" s="21" customFormat="1" ht="21.75">
-      <c r="A83" s="189"/>
-      <c r="B83" s="153"/>
-      <c r="C83" s="122"/>
+      <c r="A83" s="148"/>
+      <c r="B83" s="191"/>
+      <c r="C83" s="193"/>
       <c r="D83" s="80" t="s">
         <v>144</v>
       </c>
@@ -4651,15 +4651,15 @@
       </c>
       <c r="G83" s="109"/>
       <c r="H83" s="110"/>
-      <c r="I83" s="151"/>
-      <c r="J83" s="120"/>
-      <c r="K83" s="120"/>
-      <c r="L83" s="151"/>
+      <c r="I83" s="179"/>
+      <c r="J83" s="174"/>
+      <c r="K83" s="174"/>
+      <c r="L83" s="179"/>
     </row>
     <row r="84" spans="1:12" s="21" customFormat="1" ht="20.100000000000001">
-      <c r="A84" s="189"/>
-      <c r="B84" s="153"/>
-      <c r="C84" s="122"/>
+      <c r="A84" s="148"/>
+      <c r="B84" s="191"/>
+      <c r="C84" s="193"/>
       <c r="D84" s="80" t="s">
         <v>145</v>
       </c>
@@ -4671,15 +4671,15 @@
       </c>
       <c r="G84" s="109"/>
       <c r="H84" s="110"/>
-      <c r="I84" s="152"/>
-      <c r="J84" s="121"/>
-      <c r="K84" s="121"/>
-      <c r="L84" s="152"/>
+      <c r="I84" s="190"/>
+      <c r="J84" s="175"/>
+      <c r="K84" s="175"/>
+      <c r="L84" s="190"/>
     </row>
     <row r="85" spans="1:12" s="21" customFormat="1" ht="20.100000000000001">
-      <c r="A85" s="189"/>
-      <c r="B85" s="153"/>
-      <c r="C85" s="122"/>
+      <c r="A85" s="148"/>
+      <c r="B85" s="191"/>
+      <c r="C85" s="193"/>
       <c r="D85" s="80" t="s">
         <v>147</v>
       </c>
@@ -4691,19 +4691,19 @@
       </c>
       <c r="G85" s="109"/>
       <c r="H85" s="110"/>
-      <c r="I85" s="150"/>
-      <c r="J85" s="119" t="s">
+      <c r="I85" s="189"/>
+      <c r="J85" s="173" t="s">
         <v>149</v>
       </c>
-      <c r="K85" s="119" t="s">
+      <c r="K85" s="173" t="s">
         <v>150</v>
       </c>
-      <c r="L85" s="150"/>
+      <c r="L85" s="189"/>
     </row>
     <row r="86" spans="1:12" s="21" customFormat="1" ht="20.100000000000001">
-      <c r="A86" s="189"/>
-      <c r="B86" s="153"/>
-      <c r="C86" s="122"/>
+      <c r="A86" s="148"/>
+      <c r="B86" s="191"/>
+      <c r="C86" s="193"/>
       <c r="D86" s="80" t="s">
         <v>151</v>
       </c>
@@ -4715,15 +4715,15 @@
       </c>
       <c r="G86" s="109"/>
       <c r="H86" s="110"/>
-      <c r="I86" s="152"/>
-      <c r="J86" s="121"/>
-      <c r="K86" s="121"/>
-      <c r="L86" s="152"/>
+      <c r="I86" s="190"/>
+      <c r="J86" s="175"/>
+      <c r="K86" s="175"/>
+      <c r="L86" s="190"/>
     </row>
     <row r="87" spans="1:12" s="21" customFormat="1">
-      <c r="A87" s="189"/>
-      <c r="B87" s="153"/>
-      <c r="C87" s="122"/>
+      <c r="A87" s="148"/>
+      <c r="B87" s="191"/>
+      <c r="C87" s="193"/>
       <c r="D87" s="80" t="s">
         <v>152</v>
       </c>
@@ -4734,15 +4734,15 @@
       <c r="G87" s="109"/>
       <c r="H87" s="110"/>
       <c r="I87" s="75"/>
-      <c r="J87" s="119" t="s">
+      <c r="J87" s="173" t="s">
         <v>87</v>
       </c>
       <c r="K87" s="75"/>
       <c r="L87" s="111"/>
     </row>
     <row r="88" spans="1:12">
-      <c r="A88" s="189"/>
-      <c r="B88" s="153"/>
+      <c r="A88" s="148"/>
+      <c r="B88" s="191"/>
       <c r="C88" s="48" t="s">
         <v>27</v>
       </c>
@@ -4756,13 +4756,13 @@
       <c r="G88" s="7"/>
       <c r="H88" s="31"/>
       <c r="I88" s="10"/>
-      <c r="J88" s="120"/>
+      <c r="J88" s="174"/>
       <c r="K88" s="15"/>
       <c r="L88" s="12"/>
     </row>
     <row r="89" spans="1:12" ht="64.5">
-      <c r="A89" s="190"/>
-      <c r="B89" s="153"/>
+      <c r="A89" s="149"/>
+      <c r="B89" s="191"/>
       <c r="C89" s="48" t="s">
         <v>27</v>
       </c>
@@ -4778,36 +4778,36 @@
       <c r="I89" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="J89" s="121"/>
+      <c r="J89" s="175"/>
       <c r="K89" s="10"/>
       <c r="L89" s="8"/>
     </row>
-    <row r="90" spans="1:12" s="21" customFormat="1" ht="10.5">
-      <c r="A90" s="199" t="s">
+    <row r="90" spans="1:12" s="21" customFormat="1" ht="10.5" customHeight="1">
+      <c r="A90" s="160" t="s">
         <v>157</v>
       </c>
-      <c r="B90" s="146" t="s">
+      <c r="B90" s="186" t="s">
         <v>158</v>
       </c>
-      <c r="C90" s="147"/>
-      <c r="D90" s="147"/>
-      <c r="E90" s="147"/>
-      <c r="F90" s="148"/>
+      <c r="C90" s="187"/>
+      <c r="D90" s="187"/>
+      <c r="E90" s="187"/>
+      <c r="F90" s="188"/>
       <c r="G90" s="83"/>
       <c r="H90" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="I90" s="175"/>
-      <c r="J90" s="176"/>
-      <c r="K90" s="176"/>
-      <c r="L90" s="177"/>
+      <c r="I90" s="134"/>
+      <c r="J90" s="135"/>
+      <c r="K90" s="135"/>
+      <c r="L90" s="136"/>
     </row>
     <row r="91" spans="1:12" s="21" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A91" s="200"/>
-      <c r="B91" s="149" t="s">
+      <c r="A91" s="161"/>
+      <c r="B91" s="156" t="s">
         <v>159</v>
       </c>
-      <c r="C91" s="119" t="s">
+      <c r="C91" s="173" t="s">
         <v>139</v>
       </c>
       <c r="D91" s="75" t="s">
@@ -4821,19 +4821,19 @@
       </c>
       <c r="G91" s="109"/>
       <c r="H91" s="75"/>
-      <c r="I91" s="119"/>
-      <c r="J91" s="119" t="s">
+      <c r="I91" s="173"/>
+      <c r="J91" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="K91" s="119" t="s">
+      <c r="K91" s="173" t="s">
         <v>143</v>
       </c>
-      <c r="L91" s="150"/>
+      <c r="L91" s="189"/>
     </row>
     <row r="92" spans="1:12" s="21" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A92" s="200"/>
-      <c r="B92" s="125"/>
-      <c r="C92" s="120"/>
+      <c r="A92" s="161"/>
+      <c r="B92" s="157"/>
+      <c r="C92" s="174"/>
       <c r="D92" s="75" t="s">
         <v>161</v>
       </c>
@@ -4845,15 +4845,15 @@
       </c>
       <c r="G92" s="109"/>
       <c r="H92" s="75"/>
-      <c r="I92" s="120"/>
-      <c r="J92" s="120"/>
-      <c r="K92" s="120"/>
-      <c r="L92" s="151"/>
+      <c r="I92" s="174"/>
+      <c r="J92" s="174"/>
+      <c r="K92" s="174"/>
+      <c r="L92" s="179"/>
     </row>
     <row r="93" spans="1:12" s="21" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A93" s="200"/>
-      <c r="B93" s="125"/>
-      <c r="C93" s="120"/>
+      <c r="A93" s="161"/>
+      <c r="B93" s="157"/>
+      <c r="C93" s="174"/>
       <c r="D93" s="75" t="s">
         <v>162</v>
       </c>
@@ -4865,15 +4865,15 @@
       </c>
       <c r="G93" s="109"/>
       <c r="H93" s="75"/>
-      <c r="I93" s="121"/>
-      <c r="J93" s="121"/>
-      <c r="K93" s="121"/>
-      <c r="L93" s="152"/>
+      <c r="I93" s="175"/>
+      <c r="J93" s="175"/>
+      <c r="K93" s="175"/>
+      <c r="L93" s="190"/>
     </row>
     <row r="94" spans="1:12" s="21" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A94" s="200"/>
-      <c r="B94" s="125"/>
-      <c r="C94" s="120"/>
+      <c r="A94" s="161"/>
+      <c r="B94" s="157"/>
+      <c r="C94" s="174"/>
       <c r="D94" s="75" t="s">
         <v>163</v>
       </c>
@@ -4885,19 +4885,19 @@
       </c>
       <c r="G94" s="109"/>
       <c r="H94" s="75"/>
-      <c r="I94" s="119"/>
-      <c r="J94" s="119" t="s">
+      <c r="I94" s="173"/>
+      <c r="J94" s="173" t="s">
         <v>149</v>
       </c>
-      <c r="K94" s="119" t="s">
+      <c r="K94" s="173" t="s">
         <v>150</v>
       </c>
-      <c r="L94" s="150"/>
+      <c r="L94" s="189"/>
     </row>
     <row r="95" spans="1:12" s="21" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A95" s="200"/>
-      <c r="B95" s="125"/>
-      <c r="C95" s="120"/>
+      <c r="A95" s="161"/>
+      <c r="B95" s="157"/>
+      <c r="C95" s="174"/>
       <c r="D95" s="75" t="s">
         <v>164</v>
       </c>
@@ -4909,15 +4909,15 @@
       </c>
       <c r="G95" s="109"/>
       <c r="H95" s="75"/>
-      <c r="I95" s="121"/>
-      <c r="J95" s="121"/>
-      <c r="K95" s="121"/>
-      <c r="L95" s="152"/>
+      <c r="I95" s="175"/>
+      <c r="J95" s="175"/>
+      <c r="K95" s="175"/>
+      <c r="L95" s="190"/>
     </row>
     <row r="96" spans="1:12" ht="10.5">
-      <c r="A96" s="200"/>
-      <c r="B96" s="125"/>
-      <c r="C96" s="121"/>
+      <c r="A96" s="161"/>
+      <c r="B96" s="157"/>
+      <c r="C96" s="175"/>
       <c r="D96" s="80" t="s">
         <v>165</v>
       </c>
@@ -4928,15 +4928,15 @@
       <c r="G96" s="109"/>
       <c r="H96" s="75"/>
       <c r="I96" s="75"/>
-      <c r="J96" s="119" t="s">
+      <c r="J96" s="173" t="s">
         <v>87</v>
       </c>
       <c r="K96" s="75"/>
       <c r="L96" s="7"/>
     </row>
     <row r="97" spans="1:12" ht="9.9499999999999993" customHeight="1">
-      <c r="A97" s="200"/>
-      <c r="B97" s="125"/>
+      <c r="A97" s="161"/>
+      <c r="B97" s="157"/>
       <c r="C97" s="48" t="s">
         <v>27</v>
       </c>
@@ -4950,13 +4950,13 @@
       <c r="G97" s="7"/>
       <c r="H97" s="31"/>
       <c r="I97" s="10"/>
-      <c r="J97" s="120"/>
+      <c r="J97" s="174"/>
       <c r="K97" s="15"/>
       <c r="L97" s="12"/>
     </row>
     <row r="98" spans="1:12" ht="34.5" customHeight="1">
-      <c r="A98" s="201"/>
-      <c r="B98" s="124"/>
+      <c r="A98" s="162"/>
+      <c r="B98" s="172"/>
       <c r="C98" s="48" t="s">
         <v>27</v>
       </c>
@@ -4972,36 +4972,36 @@
       <c r="I98" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="J98" s="121"/>
+      <c r="J98" s="175"/>
       <c r="K98" s="10"/>
       <c r="L98" s="8"/>
     </row>
     <row r="99" spans="1:12" s="21" customFormat="1" ht="10.5">
-      <c r="A99" s="137" t="s">
+      <c r="A99" s="180" t="s">
         <v>170</v>
       </c>
-      <c r="B99" s="178" t="s">
+      <c r="B99" s="137" t="s">
         <v>171</v>
       </c>
-      <c r="C99" s="179"/>
-      <c r="D99" s="179"/>
-      <c r="E99" s="179"/>
-      <c r="F99" s="180"/>
+      <c r="C99" s="138"/>
+      <c r="D99" s="138"/>
+      <c r="E99" s="138"/>
+      <c r="F99" s="139"/>
       <c r="G99" s="83"/>
       <c r="H99" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="I99" s="181"/>
-      <c r="J99" s="182"/>
-      <c r="K99" s="182"/>
-      <c r="L99" s="183"/>
+      <c r="I99" s="140"/>
+      <c r="J99" s="141"/>
+      <c r="K99" s="141"/>
+      <c r="L99" s="142"/>
     </row>
     <row r="100" spans="1:12" ht="20.100000000000001">
-      <c r="A100" s="138"/>
-      <c r="B100" s="166" t="s">
+      <c r="A100" s="181"/>
+      <c r="B100" s="131" t="s">
         <v>172</v>
       </c>
-      <c r="C100" s="149" t="s">
+      <c r="C100" s="156" t="s">
         <v>91</v>
       </c>
       <c r="D100" s="80" t="s">
@@ -5016,18 +5016,18 @@
       <c r="G100" s="7"/>
       <c r="H100" s="29"/>
       <c r="I100" s="14"/>
-      <c r="J100" s="119" t="s">
+      <c r="J100" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="K100" s="119" t="s">
+      <c r="K100" s="173" t="s">
         <v>143</v>
       </c>
       <c r="L100" s="7"/>
     </row>
     <row r="101" spans="1:12" ht="20.100000000000001">
-      <c r="A101" s="138"/>
-      <c r="B101" s="167"/>
-      <c r="C101" s="125"/>
+      <c r="A101" s="181"/>
+      <c r="B101" s="132"/>
+      <c r="C101" s="157"/>
       <c r="D101" s="80" t="s">
         <v>174</v>
       </c>
@@ -5040,14 +5040,14 @@
       <c r="G101" s="7"/>
       <c r="H101" s="29"/>
       <c r="I101" s="14"/>
-      <c r="J101" s="120"/>
-      <c r="K101" s="120"/>
+      <c r="J101" s="174"/>
+      <c r="K101" s="174"/>
       <c r="L101" s="74"/>
     </row>
     <row r="102" spans="1:12" ht="20.100000000000001">
-      <c r="A102" s="138"/>
-      <c r="B102" s="167"/>
-      <c r="C102" s="125"/>
+      <c r="A102" s="181"/>
+      <c r="B102" s="132"/>
+      <c r="C102" s="157"/>
       <c r="D102" s="80" t="s">
         <v>175</v>
       </c>
@@ -5060,14 +5060,14 @@
       <c r="G102" s="7"/>
       <c r="H102" s="29"/>
       <c r="I102" s="14"/>
-      <c r="J102" s="121"/>
-      <c r="K102" s="121"/>
+      <c r="J102" s="175"/>
+      <c r="K102" s="175"/>
       <c r="L102" s="74"/>
     </row>
     <row r="103" spans="1:12" ht="20.100000000000001">
-      <c r="A103" s="138"/>
-      <c r="B103" s="167"/>
-      <c r="C103" s="125"/>
+      <c r="A103" s="181"/>
+      <c r="B103" s="132"/>
+      <c r="C103" s="157"/>
       <c r="D103" s="80" t="s">
         <v>176</v>
       </c>
@@ -5080,18 +5080,18 @@
       <c r="G103" s="7"/>
       <c r="H103" s="29"/>
       <c r="I103" s="14"/>
-      <c r="J103" s="119" t="s">
+      <c r="J103" s="173" t="s">
         <v>149</v>
       </c>
-      <c r="K103" s="119" t="s">
+      <c r="K103" s="173" t="s">
         <v>150</v>
       </c>
       <c r="L103" s="74"/>
     </row>
     <row r="104" spans="1:12" ht="20.100000000000001">
-      <c r="A104" s="138"/>
-      <c r="B104" s="167"/>
-      <c r="C104" s="125"/>
+      <c r="A104" s="181"/>
+      <c r="B104" s="132"/>
+      <c r="C104" s="157"/>
       <c r="D104" s="80" t="s">
         <v>177</v>
       </c>
@@ -5104,14 +5104,14 @@
       <c r="G104" s="7"/>
       <c r="H104" s="29"/>
       <c r="I104" s="14"/>
-      <c r="J104" s="121"/>
-      <c r="K104" s="121"/>
+      <c r="J104" s="175"/>
+      <c r="K104" s="175"/>
       <c r="L104" s="74"/>
     </row>
     <row r="105" spans="1:12">
-      <c r="A105" s="138"/>
-      <c r="B105" s="167"/>
-      <c r="C105" s="124"/>
+      <c r="A105" s="181"/>
+      <c r="B105" s="132"/>
+      <c r="C105" s="172"/>
       <c r="D105" s="80" t="s">
         <v>178</v>
       </c>
@@ -5122,15 +5122,15 @@
       <c r="G105" s="7"/>
       <c r="H105" s="29"/>
       <c r="I105" s="14"/>
-      <c r="J105" s="119" t="s">
+      <c r="J105" s="173" t="s">
         <v>87</v>
       </c>
       <c r="K105" s="75"/>
       <c r="L105" s="74"/>
     </row>
     <row r="106" spans="1:12">
-      <c r="A106" s="138"/>
-      <c r="B106" s="167"/>
+      <c r="A106" s="181"/>
+      <c r="B106" s="132"/>
       <c r="C106" s="48" t="s">
         <v>27</v>
       </c>
@@ -5144,13 +5144,13 @@
       <c r="G106" s="7"/>
       <c r="H106" s="31"/>
       <c r="I106" s="10"/>
-      <c r="J106" s="120"/>
+      <c r="J106" s="174"/>
       <c r="K106" s="15"/>
       <c r="L106" s="12"/>
     </row>
     <row r="107" spans="1:12" ht="54">
-      <c r="A107" s="139"/>
-      <c r="B107" s="168"/>
+      <c r="A107" s="182"/>
+      <c r="B107" s="133"/>
       <c r="C107" s="48" t="s">
         <v>27</v>
       </c>
@@ -5166,33 +5166,33 @@
       <c r="I107" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="J107" s="121"/>
+      <c r="J107" s="175"/>
       <c r="K107" s="10"/>
       <c r="L107" s="8"/>
     </row>
     <row r="108" spans="1:12" s="21" customFormat="1" ht="10.5" customHeight="1">
-      <c r="A108" s="140" t="s">
+      <c r="A108" s="183" t="s">
         <v>182</v>
       </c>
-      <c r="B108" s="126" t="s">
+      <c r="B108" s="199" t="s">
         <v>183</v>
       </c>
-      <c r="C108" s="127"/>
-      <c r="D108" s="127"/>
-      <c r="E108" s="128"/>
+      <c r="C108" s="200"/>
+      <c r="D108" s="200"/>
+      <c r="E108" s="201"/>
       <c r="F108" s="25"/>
       <c r="G108" s="83"/>
       <c r="H108" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I108" s="184"/>
-      <c r="J108" s="185"/>
-      <c r="K108" s="185"/>
-      <c r="L108" s="186"/>
+      <c r="I108" s="143"/>
+      <c r="J108" s="144"/>
+      <c r="K108" s="144"/>
+      <c r="L108" s="145"/>
     </row>
     <row r="109" spans="1:12" ht="21.75">
-      <c r="A109" s="141"/>
-      <c r="B109" s="166" t="s">
+      <c r="A109" s="184"/>
+      <c r="B109" s="131" t="s">
         <v>184</v>
       </c>
       <c r="C109" s="78" t="s">
@@ -5210,17 +5210,17 @@
       <c r="G109" s="7"/>
       <c r="H109" s="29"/>
       <c r="I109" s="14"/>
-      <c r="J109" s="119" t="s">
+      <c r="J109" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="K109" s="119" t="s">
+      <c r="K109" s="173" t="s">
         <v>143</v>
       </c>
       <c r="L109" s="7"/>
     </row>
     <row r="110" spans="1:12" ht="20.100000000000001">
-      <c r="A110" s="141"/>
-      <c r="B110" s="167"/>
+      <c r="A110" s="184"/>
+      <c r="B110" s="132"/>
       <c r="C110" s="78" t="s">
         <v>27</v>
       </c>
@@ -5236,13 +5236,13 @@
       <c r="G110" s="7"/>
       <c r="H110" s="29"/>
       <c r="I110" s="14"/>
-      <c r="J110" s="120"/>
-      <c r="K110" s="120"/>
+      <c r="J110" s="174"/>
+      <c r="K110" s="174"/>
       <c r="L110" s="74"/>
     </row>
     <row r="111" spans="1:12" ht="20.100000000000001">
-      <c r="A111" s="141"/>
-      <c r="B111" s="167"/>
+      <c r="A111" s="184"/>
+      <c r="B111" s="132"/>
       <c r="C111" s="78" t="s">
         <v>27</v>
       </c>
@@ -5258,13 +5258,13 @@
       <c r="G111" s="7"/>
       <c r="H111" s="29"/>
       <c r="I111" s="14"/>
-      <c r="J111" s="121"/>
-      <c r="K111" s="121"/>
+      <c r="J111" s="175"/>
+      <c r="K111" s="175"/>
       <c r="L111" s="74"/>
     </row>
     <row r="112" spans="1:12" ht="20.100000000000001">
-      <c r="A112" s="141"/>
-      <c r="B112" s="167"/>
+      <c r="A112" s="184"/>
+      <c r="B112" s="132"/>
       <c r="C112" s="78" t="s">
         <v>27</v>
       </c>
@@ -5280,17 +5280,17 @@
       <c r="G112" s="7"/>
       <c r="H112" s="29"/>
       <c r="I112" s="14"/>
-      <c r="J112" s="119" t="s">
+      <c r="J112" s="173" t="s">
         <v>149</v>
       </c>
-      <c r="K112" s="119" t="s">
+      <c r="K112" s="173" t="s">
         <v>150</v>
       </c>
       <c r="L112" s="74"/>
     </row>
     <row r="113" spans="1:12" ht="20.100000000000001">
-      <c r="A113" s="141"/>
-      <c r="B113" s="167"/>
+      <c r="A113" s="184"/>
+      <c r="B113" s="132"/>
       <c r="C113" s="78" t="s">
         <v>27</v>
       </c>
@@ -5306,13 +5306,13 @@
       <c r="G113" s="7"/>
       <c r="H113" s="29"/>
       <c r="I113" s="14"/>
-      <c r="J113" s="121"/>
-      <c r="K113" s="121"/>
+      <c r="J113" s="175"/>
+      <c r="K113" s="175"/>
       <c r="L113" s="74"/>
     </row>
     <row r="114" spans="1:12">
-      <c r="A114" s="141"/>
-      <c r="B114" s="167"/>
+      <c r="A114" s="184"/>
+      <c r="B114" s="132"/>
       <c r="C114" s="78" t="s">
         <v>27</v>
       </c>
@@ -5326,15 +5326,15 @@
       <c r="G114" s="7"/>
       <c r="H114" s="29"/>
       <c r="I114" s="14"/>
-      <c r="J114" s="119" t="s">
+      <c r="J114" s="173" t="s">
         <v>87</v>
       </c>
       <c r="K114" s="75"/>
       <c r="L114" s="74"/>
     </row>
     <row r="115" spans="1:12">
-      <c r="A115" s="141"/>
-      <c r="B115" s="167"/>
+      <c r="A115" s="184"/>
+      <c r="B115" s="132"/>
       <c r="C115" s="48" t="s">
         <v>27</v>
       </c>
@@ -5348,13 +5348,13 @@
       <c r="G115" s="10"/>
       <c r="H115" s="31"/>
       <c r="I115" s="10"/>
-      <c r="J115" s="120"/>
+      <c r="J115" s="174"/>
       <c r="K115" s="15"/>
       <c r="L115" s="12"/>
     </row>
     <row r="116" spans="1:12">
-      <c r="A116" s="142"/>
-      <c r="B116" s="168"/>
+      <c r="A116" s="185"/>
+      <c r="B116" s="133"/>
       <c r="C116" s="48" t="s">
         <v>27</v>
       </c>
@@ -5370,15 +5370,15 @@
       <c r="I116" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="J116" s="121"/>
+      <c r="J116" s="175"/>
       <c r="K116" s="10"/>
       <c r="L116" s="8"/>
     </row>
     <row r="117" spans="1:12" ht="10.5">
-      <c r="A117" s="198" t="s">
+      <c r="A117" s="159" t="s">
         <v>194</v>
       </c>
-      <c r="B117" s="166" t="s">
+      <c r="B117" s="131" t="s">
         <v>195</v>
       </c>
       <c r="C117" s="48" t="s">
@@ -5401,8 +5401,8 @@
       <c r="L117" s="10"/>
     </row>
     <row r="118" spans="1:12" ht="10.5">
-      <c r="A118" s="198"/>
-      <c r="B118" s="167"/>
+      <c r="A118" s="159"/>
+      <c r="B118" s="132"/>
       <c r="C118" s="48" t="s">
         <v>27</v>
       </c>
@@ -5421,8 +5421,8 @@
       <c r="L118" s="10"/>
     </row>
     <row r="119" spans="1:12">
-      <c r="A119" s="198"/>
-      <c r="B119" s="167"/>
+      <c r="A119" s="159"/>
+      <c r="B119" s="132"/>
       <c r="C119" s="48" t="s">
         <v>27</v>
       </c>
@@ -5441,8 +5441,8 @@
       <c r="L119" s="10"/>
     </row>
     <row r="120" spans="1:12">
-      <c r="A120" s="198"/>
-      <c r="B120" s="167"/>
+      <c r="A120" s="159"/>
+      <c r="B120" s="132"/>
       <c r="C120" s="48" t="s">
         <v>199</v>
       </c>
@@ -5461,8 +5461,8 @@
       <c r="L120" s="10"/>
     </row>
     <row r="121" spans="1:12">
-      <c r="A121" s="198"/>
-      <c r="B121" s="168"/>
+      <c r="A121" s="159"/>
+      <c r="B121" s="133"/>
       <c r="C121" s="48" t="s">
         <v>199</v>
       </c>
@@ -5481,7 +5481,7 @@
       <c r="L121" s="10"/>
     </row>
     <row r="122" spans="1:12">
-      <c r="A122" s="197"/>
+      <c r="A122" s="158"/>
       <c r="B122" s="56"/>
       <c r="C122" s="57" t="s">
         <v>24</v>
@@ -5501,24 +5501,24 @@
       <c r="L122" s="53"/>
     </row>
     <row r="123" spans="1:12" s="21" customFormat="1" ht="10.5">
-      <c r="A123" s="197"/>
-      <c r="B123" s="143" t="s">
+      <c r="A123" s="158"/>
+      <c r="B123" s="128" t="s">
         <v>204</v>
       </c>
-      <c r="C123" s="144"/>
-      <c r="D123" s="144"/>
-      <c r="E123" s="144"/>
-      <c r="F123" s="145"/>
+      <c r="C123" s="129"/>
+      <c r="D123" s="129"/>
+      <c r="E123" s="129"/>
+      <c r="F123" s="130"/>
       <c r="G123" s="83"/>
       <c r="H123" s="28"/>
-      <c r="I123" s="172"/>
-      <c r="J123" s="173"/>
-      <c r="K123" s="173"/>
-      <c r="L123" s="174"/>
+      <c r="I123" s="125"/>
+      <c r="J123" s="126"/>
+      <c r="K123" s="126"/>
+      <c r="L123" s="127"/>
     </row>
     <row r="124" spans="1:12">
-      <c r="A124" s="161"/>
-      <c r="B124" s="168" t="s">
+      <c r="A124" s="120"/>
+      <c r="B124" s="133" t="s">
         <v>205</v>
       </c>
       <c r="C124" s="48" t="s">
@@ -5541,8 +5541,8 @@
       <c r="L124" s="20"/>
     </row>
     <row r="125" spans="1:12" ht="20.100000000000001">
-      <c r="A125" s="161"/>
-      <c r="B125" s="168"/>
+      <c r="A125" s="120"/>
+      <c r="B125" s="133"/>
       <c r="C125" s="48"/>
       <c r="D125" s="75" t="s">
         <v>207</v>
@@ -5556,17 +5556,17 @@
       <c r="G125" s="20"/>
       <c r="H125" s="33"/>
       <c r="I125" s="20"/>
-      <c r="J125" s="119" t="s">
+      <c r="J125" s="173" t="s">
         <v>142</v>
       </c>
-      <c r="K125" s="119" t="s">
+      <c r="K125" s="173" t="s">
         <v>208</v>
       </c>
       <c r="L125" s="20"/>
     </row>
     <row r="126" spans="1:12" ht="20.100000000000001">
-      <c r="A126" s="161"/>
-      <c r="B126" s="168"/>
+      <c r="A126" s="120"/>
+      <c r="B126" s="133"/>
       <c r="C126" s="48"/>
       <c r="D126" s="75" t="s">
         <v>209</v>
@@ -5580,13 +5580,13 @@
       <c r="G126" s="20"/>
       <c r="H126" s="33"/>
       <c r="I126" s="20"/>
-      <c r="J126" s="125"/>
-      <c r="K126" s="120"/>
+      <c r="J126" s="157"/>
+      <c r="K126" s="174"/>
       <c r="L126" s="20"/>
     </row>
     <row r="127" spans="1:12" ht="20.100000000000001">
-      <c r="A127" s="161"/>
-      <c r="B127" s="168"/>
+      <c r="A127" s="120"/>
+      <c r="B127" s="133"/>
       <c r="C127" s="48"/>
       <c r="D127" s="75" t="s">
         <v>210</v>
@@ -5600,13 +5600,13 @@
       <c r="G127" s="20"/>
       <c r="H127" s="33"/>
       <c r="I127" s="20"/>
-      <c r="J127" s="124"/>
-      <c r="K127" s="121"/>
+      <c r="J127" s="172"/>
+      <c r="K127" s="175"/>
       <c r="L127" s="20"/>
     </row>
     <row r="128" spans="1:12" ht="20.100000000000001">
-      <c r="A128" s="161"/>
-      <c r="B128" s="168"/>
+      <c r="A128" s="120"/>
+      <c r="B128" s="133"/>
       <c r="C128" s="48"/>
       <c r="D128" s="75" t="s">
         <v>211</v>
@@ -5620,17 +5620,17 @@
       <c r="G128" s="20"/>
       <c r="H128" s="33"/>
       <c r="I128" s="20"/>
-      <c r="J128" s="119" t="s">
+      <c r="J128" s="173" t="s">
         <v>149</v>
       </c>
-      <c r="K128" s="119" t="s">
+      <c r="K128" s="173" t="s">
         <v>150</v>
       </c>
       <c r="L128" s="20"/>
     </row>
     <row r="129" spans="1:12" ht="20.100000000000001">
-      <c r="A129" s="161"/>
-      <c r="B129" s="168"/>
+      <c r="A129" s="120"/>
+      <c r="B129" s="133"/>
       <c r="C129" s="48"/>
       <c r="D129" s="75" t="s">
         <v>212</v>
@@ -5644,13 +5644,13 @@
       <c r="G129" s="20"/>
       <c r="H129" s="33"/>
       <c r="I129" s="20"/>
-      <c r="J129" s="124"/>
-      <c r="K129" s="124"/>
+      <c r="J129" s="172"/>
+      <c r="K129" s="172"/>
       <c r="L129" s="20"/>
     </row>
     <row r="130" spans="1:12">
-      <c r="A130" s="161"/>
-      <c r="B130" s="187"/>
+      <c r="A130" s="120"/>
+      <c r="B130" s="146"/>
       <c r="C130" s="8" t="s">
         <v>91</v>
       </c>
@@ -5671,8 +5671,8 @@
       <c r="L130" s="10"/>
     </row>
     <row r="131" spans="1:12">
-      <c r="A131" s="162"/>
-      <c r="B131" s="187"/>
+      <c r="A131" s="121"/>
+      <c r="B131" s="146"/>
       <c r="C131" s="48" t="s">
         <v>27</v>
       </c>
@@ -5691,7 +5691,7 @@
       <c r="L131" s="10"/>
     </row>
     <row r="132" spans="1:12">
-      <c r="A132" s="160" t="s">
+      <c r="A132" s="119" t="s">
         <v>215</v>
       </c>
       <c r="B132" s="56"/>
@@ -5713,8 +5713,8 @@
       <c r="L132" s="53"/>
     </row>
     <row r="133" spans="1:12">
-      <c r="A133" s="161"/>
-      <c r="B133" s="122" t="s">
+      <c r="A133" s="120"/>
+      <c r="B133" s="193" t="s">
         <v>216</v>
       </c>
       <c r="C133" s="11" t="s">
@@ -5737,8 +5737,8 @@
       <c r="L133" s="10"/>
     </row>
     <row r="134" spans="1:12">
-      <c r="A134" s="161"/>
-      <c r="B134" s="122"/>
+      <c r="A134" s="120"/>
+      <c r="B134" s="193"/>
       <c r="C134" s="11" t="s">
         <v>27</v>
       </c>
@@ -5757,8 +5757,8 @@
       <c r="L134" s="10"/>
     </row>
     <row r="135" spans="1:12">
-      <c r="A135" s="161"/>
-      <c r="B135" s="122"/>
+      <c r="A135" s="120"/>
+      <c r="B135" s="193"/>
       <c r="C135" s="8" t="s">
         <v>27</v>
       </c>
@@ -5777,8 +5777,8 @@
       <c r="L135" s="8"/>
     </row>
     <row r="136" spans="1:12">
-      <c r="A136" s="161"/>
-      <c r="B136" s="122"/>
+      <c r="A136" s="120"/>
+      <c r="B136" s="193"/>
       <c r="C136" s="8" t="s">
         <v>27</v>
       </c>
@@ -5797,9 +5797,9 @@
       <c r="L136" s="10"/>
     </row>
     <row r="137" spans="1:12" ht="20.100000000000001">
-      <c r="A137" s="162"/>
-      <c r="B137" s="122"/>
-      <c r="C137" s="122" t="s">
+      <c r="A137" s="121"/>
+      <c r="B137" s="193"/>
+      <c r="C137" s="193" t="s">
         <v>91</v>
       </c>
       <c r="D137" s="75" t="s">
@@ -5814,18 +5814,18 @@
       <c r="G137" s="7"/>
       <c r="H137" s="31"/>
       <c r="I137" s="10"/>
-      <c r="J137" s="123" t="s">
+      <c r="J137" s="192" t="s">
         <v>142</v>
       </c>
-      <c r="K137" s="123" t="s">
+      <c r="K137" s="192" t="s">
         <v>143</v>
       </c>
       <c r="L137" s="10"/>
     </row>
     <row r="138" spans="1:12" ht="20.100000000000001">
       <c r="A138" s="62"/>
-      <c r="B138" s="122"/>
-      <c r="C138" s="122"/>
+      <c r="B138" s="193"/>
+      <c r="C138" s="193"/>
       <c r="D138" s="75" t="s">
         <v>222</v>
       </c>
@@ -5838,14 +5838,14 @@
       <c r="G138" s="7"/>
       <c r="H138" s="31"/>
       <c r="I138" s="10"/>
-      <c r="J138" s="122"/>
-      <c r="K138" s="122"/>
+      <c r="J138" s="193"/>
+      <c r="K138" s="193"/>
       <c r="L138" s="10"/>
     </row>
     <row r="139" spans="1:12" ht="20.100000000000001">
       <c r="A139" s="62"/>
-      <c r="B139" s="122"/>
-      <c r="C139" s="122"/>
+      <c r="B139" s="193"/>
+      <c r="C139" s="193"/>
       <c r="D139" s="75" t="s">
         <v>223</v>
       </c>
@@ -5858,14 +5858,14 @@
       <c r="G139" s="7"/>
       <c r="H139" s="31"/>
       <c r="I139" s="10"/>
-      <c r="J139" s="122"/>
-      <c r="K139" s="122"/>
+      <c r="J139" s="193"/>
+      <c r="K139" s="193"/>
       <c r="L139" s="10"/>
     </row>
     <row r="140" spans="1:12" ht="20.100000000000001">
       <c r="A140" s="62"/>
-      <c r="B140" s="122"/>
-      <c r="C140" s="122"/>
+      <c r="B140" s="193"/>
+      <c r="C140" s="193"/>
       <c r="D140" s="75" t="s">
         <v>224</v>
       </c>
@@ -5878,18 +5878,18 @@
       <c r="G140" s="7"/>
       <c r="H140" s="31"/>
       <c r="I140" s="10"/>
-      <c r="J140" s="123" t="s">
+      <c r="J140" s="192" t="s">
         <v>149</v>
       </c>
-      <c r="K140" s="123" t="s">
+      <c r="K140" s="192" t="s">
         <v>150</v>
       </c>
       <c r="L140" s="10"/>
     </row>
     <row r="141" spans="1:12" ht="20.100000000000001">
       <c r="A141" s="62"/>
-      <c r="B141" s="122"/>
-      <c r="C141" s="122"/>
+      <c r="B141" s="193"/>
+      <c r="C141" s="193"/>
       <c r="D141" s="75" t="s">
         <v>225</v>
       </c>
@@ -5902,14 +5902,14 @@
       <c r="G141" s="7"/>
       <c r="H141" s="31"/>
       <c r="I141" s="10"/>
-      <c r="J141" s="122"/>
-      <c r="K141" s="122"/>
+      <c r="J141" s="193"/>
+      <c r="K141" s="193"/>
       <c r="L141" s="10"/>
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="62"/>
-      <c r="B142" s="122"/>
-      <c r="C142" s="122"/>
+      <c r="B142" s="193"/>
+      <c r="C142" s="193"/>
       <c r="D142" s="75" t="s">
         <v>226</v>
       </c>
@@ -5927,7 +5927,7 @@
       <c r="L142" s="10"/>
     </row>
     <row r="143" spans="1:12">
-      <c r="A143" s="160" t="s">
+      <c r="A143" s="119" t="s">
         <v>227</v>
       </c>
       <c r="B143" s="38"/>
@@ -5947,8 +5947,8 @@
       <c r="L143" s="44"/>
     </row>
     <row r="144" spans="1:12" ht="10.5">
-      <c r="A144" s="161"/>
-      <c r="B144" s="170" t="s">
+      <c r="A144" s="120"/>
+      <c r="B144" s="122" t="s">
         <v>227</v>
       </c>
       <c r="C144" s="18"/>
@@ -5967,8 +5967,8 @@
       <c r="L144" s="10"/>
     </row>
     <row r="145" spans="1:12">
-      <c r="A145" s="161"/>
-      <c r="B145" s="171"/>
+      <c r="A145" s="120"/>
+      <c r="B145" s="123"/>
       <c r="C145" s="48" t="s">
         <v>27</v>
       </c>
@@ -5989,8 +5989,8 @@
       <c r="L145" s="10"/>
     </row>
     <row r="146" spans="1:12">
-      <c r="A146" s="161"/>
-      <c r="B146" s="171"/>
+      <c r="A146" s="120"/>
+      <c r="B146" s="123"/>
       <c r="C146" s="48" t="s">
         <v>27</v>
       </c>
@@ -6011,8 +6011,8 @@
       <c r="L146" s="10"/>
     </row>
     <row r="147" spans="1:12">
-      <c r="A147" s="161"/>
-      <c r="B147" s="171"/>
+      <c r="A147" s="120"/>
+      <c r="B147" s="123"/>
       <c r="C147" s="48" t="s">
         <v>27</v>
       </c>
@@ -6033,8 +6033,8 @@
       <c r="L147" s="10"/>
     </row>
     <row r="148" spans="1:12">
-      <c r="A148" s="161"/>
-      <c r="B148" s="171"/>
+      <c r="A148" s="120"/>
+      <c r="B148" s="123"/>
       <c r="C148" s="48" t="s">
         <v>27</v>
       </c>
@@ -6055,8 +6055,8 @@
       <c r="L148" s="10"/>
     </row>
     <row r="149" spans="1:12">
-      <c r="A149" s="161"/>
-      <c r="B149" s="171"/>
+      <c r="A149" s="120"/>
+      <c r="B149" s="123"/>
       <c r="C149" s="48" t="s">
         <v>27</v>
       </c>
@@ -6077,8 +6077,8 @@
       <c r="L149" s="10"/>
     </row>
     <row r="150" spans="1:12">
-      <c r="A150" s="161"/>
-      <c r="B150" s="171"/>
+      <c r="A150" s="120"/>
+      <c r="B150" s="123"/>
       <c r="C150" s="48" t="s">
         <v>27</v>
       </c>
@@ -6099,8 +6099,8 @@
       <c r="L150" s="10"/>
     </row>
     <row r="151" spans="1:12">
-      <c r="A151" s="161"/>
-      <c r="B151" s="171"/>
+      <c r="A151" s="120"/>
+      <c r="B151" s="123"/>
       <c r="C151" s="48" t="s">
         <v>27</v>
       </c>
@@ -6121,8 +6121,8 @@
       <c r="L151" s="10"/>
     </row>
     <row r="152" spans="1:12">
-      <c r="A152" s="162"/>
-      <c r="B152" s="169"/>
+      <c r="A152" s="121"/>
+      <c r="B152" s="124"/>
       <c r="C152" s="48" t="s">
         <v>27</v>
       </c>
@@ -6164,6 +6164,95 @@
     </row>
   </sheetData>
   <mergeCells count="113">
+    <mergeCell ref="J105:J107"/>
+    <mergeCell ref="J114:J116"/>
+    <mergeCell ref="C137:C142"/>
+    <mergeCell ref="B133:B142"/>
+    <mergeCell ref="J137:J139"/>
+    <mergeCell ref="K137:K139"/>
+    <mergeCell ref="J140:J141"/>
+    <mergeCell ref="K140:K141"/>
+    <mergeCell ref="J109:J111"/>
+    <mergeCell ref="J112:J113"/>
+    <mergeCell ref="K109:K111"/>
+    <mergeCell ref="K112:K113"/>
+    <mergeCell ref="K125:K127"/>
+    <mergeCell ref="K128:K129"/>
+    <mergeCell ref="J125:J127"/>
+    <mergeCell ref="J128:J129"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="K100:K102"/>
+    <mergeCell ref="K103:K104"/>
+    <mergeCell ref="J100:J102"/>
+    <mergeCell ref="J103:J104"/>
+    <mergeCell ref="K36:K38"/>
+    <mergeCell ref="K39:K40"/>
+    <mergeCell ref="I43:I48"/>
+    <mergeCell ref="J43:J45"/>
+    <mergeCell ref="K43:K45"/>
+    <mergeCell ref="J46:J47"/>
+    <mergeCell ref="K46:K47"/>
+    <mergeCell ref="J87:J89"/>
+    <mergeCell ref="J96:J98"/>
+    <mergeCell ref="C82:C87"/>
+    <mergeCell ref="I62:I67"/>
+    <mergeCell ref="J62:J64"/>
+    <mergeCell ref="J65:J66"/>
+    <mergeCell ref="K62:K64"/>
+    <mergeCell ref="K65:K66"/>
+    <mergeCell ref="C69:C74"/>
+    <mergeCell ref="I69:I74"/>
+    <mergeCell ref="J69:J71"/>
+    <mergeCell ref="K69:K71"/>
+    <mergeCell ref="J72:J73"/>
+    <mergeCell ref="K72:K73"/>
+    <mergeCell ref="A99:A107"/>
+    <mergeCell ref="A108:A116"/>
+    <mergeCell ref="B123:F123"/>
+    <mergeCell ref="B90:F90"/>
+    <mergeCell ref="C100:C105"/>
+    <mergeCell ref="L82:L84"/>
+    <mergeCell ref="L85:L86"/>
+    <mergeCell ref="B91:B98"/>
+    <mergeCell ref="C91:C96"/>
+    <mergeCell ref="I91:I93"/>
+    <mergeCell ref="I94:I95"/>
+    <mergeCell ref="K91:K93"/>
+    <mergeCell ref="J91:J93"/>
+    <mergeCell ref="J94:J95"/>
+    <mergeCell ref="K94:K95"/>
+    <mergeCell ref="L91:L93"/>
+    <mergeCell ref="L94:L95"/>
+    <mergeCell ref="J82:J84"/>
+    <mergeCell ref="J85:J86"/>
+    <mergeCell ref="K82:K84"/>
+    <mergeCell ref="K85:K86"/>
+    <mergeCell ref="I82:I84"/>
+    <mergeCell ref="I85:I86"/>
+    <mergeCell ref="B82:B89"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:A18"/>
+    <mergeCell ref="A19:A27"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="B20:B27"/>
+    <mergeCell ref="B30:B54"/>
+    <mergeCell ref="C56:C61"/>
+    <mergeCell ref="J59:J60"/>
+    <mergeCell ref="J56:J58"/>
+    <mergeCell ref="K56:K58"/>
+    <mergeCell ref="K59:K60"/>
+    <mergeCell ref="I56:I61"/>
+    <mergeCell ref="C30:C35"/>
+    <mergeCell ref="I36:I41"/>
+    <mergeCell ref="J36:J38"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="I30:I35"/>
+    <mergeCell ref="J30:J32"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="K30:K32"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="C36:C41"/>
+    <mergeCell ref="C43:C48"/>
     <mergeCell ref="A143:A152"/>
     <mergeCell ref="B144:B152"/>
     <mergeCell ref="I123:L123"/>
@@ -6188,95 +6277,6 @@
     <mergeCell ref="B109:B116"/>
     <mergeCell ref="B117:B121"/>
     <mergeCell ref="A90:A98"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A4:A18"/>
-    <mergeCell ref="A19:A27"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B30:B54"/>
-    <mergeCell ref="C56:C61"/>
-    <mergeCell ref="J59:J60"/>
-    <mergeCell ref="J56:J58"/>
-    <mergeCell ref="K56:K58"/>
-    <mergeCell ref="K59:K60"/>
-    <mergeCell ref="I56:I61"/>
-    <mergeCell ref="C30:C35"/>
-    <mergeCell ref="I36:I41"/>
-    <mergeCell ref="J36:J38"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="I30:I35"/>
-    <mergeCell ref="J30:J32"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="K30:K32"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="C36:C41"/>
-    <mergeCell ref="C43:C48"/>
-    <mergeCell ref="A99:A107"/>
-    <mergeCell ref="A108:A116"/>
-    <mergeCell ref="B123:F123"/>
-    <mergeCell ref="B90:F90"/>
-    <mergeCell ref="C100:C105"/>
-    <mergeCell ref="L82:L84"/>
-    <mergeCell ref="L85:L86"/>
-    <mergeCell ref="B91:B98"/>
-    <mergeCell ref="C91:C96"/>
-    <mergeCell ref="I91:I93"/>
-    <mergeCell ref="I94:I95"/>
-    <mergeCell ref="K91:K93"/>
-    <mergeCell ref="J91:J93"/>
-    <mergeCell ref="J94:J95"/>
-    <mergeCell ref="K94:K95"/>
-    <mergeCell ref="L91:L93"/>
-    <mergeCell ref="L94:L95"/>
-    <mergeCell ref="J82:J84"/>
-    <mergeCell ref="J85:J86"/>
-    <mergeCell ref="K82:K84"/>
-    <mergeCell ref="K85:K86"/>
-    <mergeCell ref="I82:I84"/>
-    <mergeCell ref="I85:I86"/>
-    <mergeCell ref="B82:B89"/>
-    <mergeCell ref="C82:C87"/>
-    <mergeCell ref="I62:I67"/>
-    <mergeCell ref="J62:J64"/>
-    <mergeCell ref="J65:J66"/>
-    <mergeCell ref="K62:K64"/>
-    <mergeCell ref="K65:K66"/>
-    <mergeCell ref="C69:C74"/>
-    <mergeCell ref="I69:I74"/>
-    <mergeCell ref="J69:J71"/>
-    <mergeCell ref="K69:K71"/>
-    <mergeCell ref="J72:J73"/>
-    <mergeCell ref="K72:K73"/>
-    <mergeCell ref="K100:K102"/>
-    <mergeCell ref="K103:K104"/>
-    <mergeCell ref="J100:J102"/>
-    <mergeCell ref="J103:J104"/>
-    <mergeCell ref="K36:K38"/>
-    <mergeCell ref="K39:K40"/>
-    <mergeCell ref="I43:I48"/>
-    <mergeCell ref="J43:J45"/>
-    <mergeCell ref="K43:K45"/>
-    <mergeCell ref="J46:J47"/>
-    <mergeCell ref="K46:K47"/>
-    <mergeCell ref="J87:J89"/>
-    <mergeCell ref="J96:J98"/>
-    <mergeCell ref="J105:J107"/>
-    <mergeCell ref="J114:J116"/>
-    <mergeCell ref="C137:C142"/>
-    <mergeCell ref="B133:B142"/>
-    <mergeCell ref="J137:J139"/>
-    <mergeCell ref="K137:K139"/>
-    <mergeCell ref="J140:J141"/>
-    <mergeCell ref="K140:K141"/>
-    <mergeCell ref="J109:J111"/>
-    <mergeCell ref="J112:J113"/>
-    <mergeCell ref="K109:K111"/>
-    <mergeCell ref="K112:K113"/>
-    <mergeCell ref="K125:K127"/>
-    <mergeCell ref="K128:K129"/>
-    <mergeCell ref="J125:J127"/>
-    <mergeCell ref="J128:J129"/>
-    <mergeCell ref="B108:E108"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7166,31 +7166,22 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <Comment xmlns="bcde6d5c-cc01-456f-b509-ecee28914122" xsi:nil="true"/>
-    <e2openHubSolution xmlns="bcde6d5c-cc01-456f-b509-ecee28914122" xsi:nil="true"/>
-    <CustomerName xmlns="bcde6d5c-cc01-456f-b509-ecee28914122" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bcde6d5c-cc01-456f-b509-ecee28914122">
+    <Comment xmlns="c71310aa-100e-4437-9936-0e26a2d7ca0b" xsi:nil="true"/>
+    <e2openHubSolution xmlns="c71310aa-100e-4437-9936-0e26a2d7ca0b" xsi:nil="true"/>
+    <CustomerName xmlns="c71310aa-100e-4437-9936-0e26a2d7ca0b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c71310aa-100e-4437-9936-0e26a2d7ca0b">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="6914a980-db16-4cd2-8b05-d07ef3ecd393" xsi:nil="true"/>
+    <TaxCatchAll xmlns="5aed2287-fa6c-4d1c-8460-e30277ab2b55" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AC747946AF76649AB026BDBC3CD52AF" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="30669be3d278a530bd7ae737eb6c6093">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bcde6d5c-cc01-456f-b509-ecee28914122" xmlns:ns3="6914a980-db16-4cd2-8b05-d07ef3ecd393" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9e65fcf57d5d8ceba4e1d7b4972c348" ns2:_="" ns3:_="">
-    <xsd:import namespace="bcde6d5c-cc01-456f-b509-ecee28914122"/>
-    <xsd:import namespace="6914a980-db16-4cd2-8b05-d07ef3ecd393"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D677334B83A01847AABB77B0676CDFF9" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="648019f14d4c62079002d151c322bf14">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c71310aa-100e-4437-9936-0e26a2d7ca0b" xmlns:ns3="5aed2287-fa6c-4d1c-8460-e30277ab2b55" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="487ba4a296563834af6b7a95f7a104cf" ns2:_="" ns3:_="">
+    <xsd:import namespace="c71310aa-100e-4437-9936-0e26a2d7ca0b"/>
+    <xsd:import namespace="5aed2287-fa6c-4d1c-8460-e30277ab2b55"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -7217,24 +7208,24 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="bcde6d5c-cc01-456f-b509-ecee28914122" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c71310aa-100e-4437-9936-0e26a2d7ca0b" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="Comment" ma:index="5" nillable="true" ma:displayName="Comment" ma:internalName="Comment" ma:readOnly="false">
+    <xsd:element name="Comment" ma:index="4" nillable="true" ma:displayName="Comment" ma:internalName="Comment" ma:readOnly="false">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="CustomerName" ma:index="7" nillable="true" ma:displayName="Customer Name" ma:description="Name of e2open 'tenant' customer" ma:internalName="CustomerName" ma:readOnly="false">
+    <xsd:element name="CustomerName" ma:index="6" nillable="true" ma:displayName="Customer Name" ma:description="Name of e2open 'tenant' customer" ma:internalName="CustomerName" ma:readOnly="false">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="e2openHubSolution" ma:index="8" nillable="true" ma:displayName="e2open Hub Solution" ma:description="Name of e2open hub solution the external party is connecting to." ma:internalName="e2openHubSolution" ma:readOnly="false">
+    <xsd:element name="e2openHubSolution" ma:index="7" nillable="true" ma:displayName="e2open Hub Solution" ma:description="Name of e2open hub solution the external party is connecting to." ma:internalName="e2openHubSolution" ma:readOnly="false">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text">
           <xsd:maxLength value="255"/>
@@ -7291,10 +7282,10 @@
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="6914a980-db16-4cd2-8b05-d07ef3ecd393" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5aed2287-fa6c-4d1c-8460-e30277ab2b55" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{045520c6-639a-4859-b252-4bab55a43234}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="6914a980-db16-4cd2-8b05-d07ef3ecd393">
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{d7fce88c-fd30-435d-8a5d-831548657414}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="5aed2287-fa6c-4d1c-8460-e30277ab2b55">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -7315,8 +7306,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="9" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="8" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="3" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -7405,14 +7396,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E06CACB8-7D8E-4511-9DC4-72EF1E1F83C6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B0855B-13ED-48DB-8B32-A648905EF182}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E677F98-5FA0-4A46-BFC1-BCB94CDFBC9E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A449C0A-4A55-403E-BF70-1D31E1491805}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7B0855B-13ED-48DB-8B32-A648905EF182}"/>
 </file>
</xml_diff>